<commit_message>
Update API tests, environment settings, package.json test scripts, and test reports
</commit_message>
<xml_diff>
--- a/Casos de prueba y reporte de bugs/Reporte de bugs.xlsx
+++ b/Casos de prueba y reporte de bugs/Reporte de bugs.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Usuario\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D14D0C8D-A2E8-4266-A373-775CDBD09A34}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E2CC5BB2-D1BB-458D-8A16-E08EA4477691}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{954EA680-8BEA-47CE-A3AB-45A46801D132}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="151" uniqueCount="67">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="175" uniqueCount="71">
   <si>
     <t>Grupo 2: Testing Exploratorio y Reporte de Bugs</t>
   </si>
@@ -298,6 +298,18 @@
   </si>
   <si>
     <t>Video de evidencia: https://1drv.ms/v/c/c95609e9bd3a56cb/IQA6RD95zzcATovuOXyUxZ4ZAR7Onq5S3Aar1K4qO9AkIJk?e=oQy4UI</t>
+  </si>
+  <si>
+    <t>Asignado</t>
+  </si>
+  <si>
+    <t>Reportado por</t>
+  </si>
+  <si>
+    <t>Thyara Vintimilla</t>
+  </si>
+  <si>
+    <t>Desarrollador X</t>
   </si>
 </sst>
 </file>
@@ -363,7 +375,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="7">
+  <borders count="8">
     <border>
       <left/>
       <right/>
@@ -449,15 +461,23 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="22">
+  <cellXfs count="23">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -484,16 +504,22 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
@@ -502,11 +528,11 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -531,13 +557,13 @@
     <xdr:from>
       <xdr:col>2</xdr:col>
       <xdr:colOff>885825</xdr:colOff>
-      <xdr:row>23</xdr:row>
+      <xdr:row>25</xdr:row>
       <xdr:rowOff>56758</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>3</xdr:col>
       <xdr:colOff>2257425</xdr:colOff>
-      <xdr:row>23</xdr:row>
+      <xdr:row>25</xdr:row>
       <xdr:rowOff>3081841</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
@@ -575,13 +601,13 @@
     <xdr:from>
       <xdr:col>6</xdr:col>
       <xdr:colOff>169621</xdr:colOff>
-      <xdr:row>23</xdr:row>
+      <xdr:row>25</xdr:row>
       <xdr:rowOff>491385</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>7</xdr:col>
       <xdr:colOff>2825204</xdr:colOff>
-      <xdr:row>23</xdr:row>
+      <xdr:row>25</xdr:row>
       <xdr:rowOff>2952750</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
@@ -619,13 +645,13 @@
     <xdr:from>
       <xdr:col>10</xdr:col>
       <xdr:colOff>391437</xdr:colOff>
-      <xdr:row>23</xdr:row>
+      <xdr:row>25</xdr:row>
       <xdr:rowOff>649115</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>11</xdr:col>
       <xdr:colOff>2560030</xdr:colOff>
-      <xdr:row>23</xdr:row>
+      <xdr:row>25</xdr:row>
       <xdr:rowOff>3048001</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
@@ -663,13 +689,13 @@
     <xdr:from>
       <xdr:col>14</xdr:col>
       <xdr:colOff>234471</xdr:colOff>
-      <xdr:row>23</xdr:row>
+      <xdr:row>25</xdr:row>
       <xdr:rowOff>666750</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>15</xdr:col>
       <xdr:colOff>2778821</xdr:colOff>
-      <xdr:row>23</xdr:row>
+      <xdr:row>25</xdr:row>
       <xdr:rowOff>2943225</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
@@ -707,13 +733,13 @@
     <xdr:from>
       <xdr:col>23</xdr:col>
       <xdr:colOff>1148714</xdr:colOff>
-      <xdr:row>23</xdr:row>
+      <xdr:row>25</xdr:row>
       <xdr:rowOff>78288</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>24</xdr:col>
       <xdr:colOff>2081493</xdr:colOff>
-      <xdr:row>23</xdr:row>
+      <xdr:row>25</xdr:row>
       <xdr:rowOff>2181226</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
@@ -751,13 +777,13 @@
     <xdr:from>
       <xdr:col>23</xdr:col>
       <xdr:colOff>1187363</xdr:colOff>
-      <xdr:row>23</xdr:row>
+      <xdr:row>25</xdr:row>
       <xdr:rowOff>1047750</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>24</xdr:col>
       <xdr:colOff>2074623</xdr:colOff>
-      <xdr:row>23</xdr:row>
+      <xdr:row>25</xdr:row>
       <xdr:rowOff>3076575</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
@@ -1091,7 +1117,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8196538F-3AA5-4A9D-BB36-23C7745390F8}">
-  <dimension ref="A2:Y24"/>
+  <dimension ref="A2:Y26"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="36.28515625" customWidth="1"/>
@@ -1109,601 +1135,709 @@
   </cols>
   <sheetData>
     <row r="2" spans="1:25" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A2" s="1" t="s">
+      <c r="A2" s="21" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="1"/>
-      <c r="C2" s="1"/>
+      <c r="B2" s="21"/>
+      <c r="C2" s="21"/>
     </row>
     <row r="3" spans="1:25" x14ac:dyDescent="0.25">
-      <c r="A3" s="2"/>
-      <c r="B3" s="2"/>
-      <c r="C3" s="2"/>
+      <c r="A3" s="1"/>
+      <c r="B3" s="1"/>
+      <c r="C3" s="1"/>
     </row>
     <row r="4" spans="1:25" x14ac:dyDescent="0.25">
-      <c r="A4" s="3" t="s">
+      <c r="A4" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="B4" s="2"/>
-      <c r="C4" s="2"/>
+      <c r="B4" s="1"/>
+      <c r="C4" s="1"/>
     </row>
     <row r="5" spans="1:25" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A5" s="2"/>
-      <c r="B5" s="2"/>
-      <c r="C5" s="4" t="s">
+      <c r="A5" s="1"/>
+      <c r="B5" s="1"/>
+      <c r="C5" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="G5" s="4" t="s">
+      <c r="G5" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="K5" s="4" t="s">
+      <c r="K5" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="O5" s="4" t="s">
+      <c r="O5" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="S5" s="4" t="s">
+      <c r="S5" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="X5" s="4" t="s">
+      <c r="X5" s="3" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="6" spans="1:25" x14ac:dyDescent="0.25">
-      <c r="A6" s="5" t="s">
+      <c r="A6" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="B6" s="2"/>
-      <c r="C6" s="2"/>
-      <c r="G6" s="2"/>
-      <c r="K6" s="2"/>
-      <c r="O6" s="2"/>
-      <c r="S6" s="2"/>
-      <c r="X6" s="2"/>
+      <c r="B6" s="1"/>
+      <c r="C6" s="1"/>
+      <c r="G6" s="1"/>
+      <c r="K6" s="1"/>
+      <c r="O6" s="1"/>
+      <c r="S6" s="1"/>
+      <c r="X6" s="1"/>
     </row>
     <row r="7" spans="1:25" x14ac:dyDescent="0.25">
-      <c r="A7" s="6" t="s">
+      <c r="A7" s="5" t="s">
         <v>9</v>
       </c>
-      <c r="B7" s="2"/>
-      <c r="C7" s="7" t="s">
+      <c r="B7" s="1"/>
+      <c r="C7" s="6" t="s">
         <v>10</v>
       </c>
-      <c r="G7" s="7" t="s">
+      <c r="G7" s="6" t="s">
         <v>11</v>
       </c>
-      <c r="K7" s="7" t="s">
+      <c r="K7" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="O7" s="7" t="s">
+      <c r="O7" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="S7" s="7" t="s">
+      <c r="S7" s="6" t="s">
         <v>14</v>
       </c>
-      <c r="X7" s="7" t="s">
+      <c r="X7" s="6" t="s">
         <v>15</v>
       </c>
     </row>
     <row r="8" spans="1:25" x14ac:dyDescent="0.25">
-      <c r="A8" s="6" t="s">
+      <c r="A8" s="5" t="s">
         <v>16</v>
       </c>
-      <c r="B8" s="2"/>
-      <c r="C8" s="2"/>
-      <c r="G8" s="2"/>
-      <c r="K8" s="2"/>
-      <c r="O8" s="2"/>
-      <c r="S8" s="2"/>
-      <c r="X8" s="2"/>
+      <c r="B8" s="1"/>
+      <c r="C8" s="1"/>
+      <c r="G8" s="1"/>
+      <c r="K8" s="1"/>
+      <c r="O8" s="1"/>
+      <c r="S8" s="1"/>
+      <c r="X8" s="1"/>
     </row>
     <row r="9" spans="1:25" x14ac:dyDescent="0.25">
-      <c r="A9" s="6" t="s">
+      <c r="A9" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="B9" s="2"/>
-      <c r="C9" s="8" t="s">
+      <c r="B9" s="1"/>
+      <c r="C9" s="7" t="s">
         <v>18</v>
       </c>
-      <c r="D9" s="8" t="s">
+      <c r="D9" s="7" t="s">
         <v>19</v>
       </c>
-      <c r="G9" s="8" t="s">
+      <c r="G9" s="7" t="s">
         <v>18</v>
       </c>
-      <c r="H9" s="8" t="s">
+      <c r="H9" s="7" t="s">
         <v>19</v>
       </c>
-      <c r="K9" s="8" t="s">
+      <c r="K9" s="7" t="s">
         <v>18</v>
       </c>
-      <c r="L9" s="8" t="s">
+      <c r="L9" s="7" t="s">
         <v>19</v>
       </c>
-      <c r="O9" s="8" t="s">
+      <c r="O9" s="7" t="s">
         <v>18</v>
       </c>
-      <c r="P9" s="8" t="s">
+      <c r="P9" s="7" t="s">
         <v>19</v>
       </c>
-      <c r="S9" s="8" t="s">
+      <c r="S9" s="7" t="s">
         <v>18</v>
       </c>
-      <c r="T9" s="8" t="s">
+      <c r="T9" s="7" t="s">
         <v>19</v>
       </c>
-      <c r="X9" s="8" t="s">
+      <c r="X9" s="7" t="s">
         <v>18</v>
       </c>
-      <c r="Y9" s="8" t="s">
+      <c r="Y9" s="7" t="s">
         <v>19</v>
       </c>
     </row>
     <row r="10" spans="1:25" x14ac:dyDescent="0.25">
-      <c r="A10" s="6" t="s">
+      <c r="A10" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="B10" s="2"/>
-      <c r="C10" s="9" t="s">
+      <c r="B10" s="1"/>
+      <c r="C10" s="8" t="s">
         <v>21</v>
       </c>
-      <c r="D10" s="10" t="s">
+      <c r="D10" s="9" t="s">
         <v>22</v>
       </c>
-      <c r="G10" s="9" t="s">
+      <c r="G10" s="8" t="s">
         <v>21</v>
       </c>
-      <c r="H10" s="10" t="s">
+      <c r="H10" s="9" t="s">
         <v>22</v>
       </c>
-      <c r="K10" s="9" t="s">
+      <c r="K10" s="8" t="s">
         <v>21</v>
       </c>
-      <c r="L10" s="10" t="s">
+      <c r="L10" s="9" t="s">
         <v>22</v>
       </c>
-      <c r="O10" s="9" t="s">
+      <c r="O10" s="8" t="s">
         <v>21</v>
       </c>
-      <c r="P10" s="10" t="s">
+      <c r="P10" s="9" t="s">
         <v>22</v>
       </c>
-      <c r="S10" s="9" t="s">
+      <c r="S10" s="8" t="s">
         <v>21</v>
       </c>
-      <c r="T10" s="10" t="s">
+      <c r="T10" s="9" t="s">
         <v>22</v>
       </c>
-      <c r="X10" s="9" t="s">
+      <c r="X10" s="8" t="s">
         <v>21</v>
       </c>
-      <c r="Y10" s="10" t="s">
+      <c r="Y10" s="9" t="s">
         <v>22</v>
       </c>
     </row>
     <row r="11" spans="1:25" x14ac:dyDescent="0.25">
-      <c r="A11" s="6" t="s">
+      <c r="A11" s="5" t="s">
         <v>23</v>
       </c>
-      <c r="B11" s="2"/>
-      <c r="C11" s="9" t="s">
+      <c r="B11" s="1"/>
+      <c r="C11" s="8" t="s">
         <v>24</v>
       </c>
-      <c r="D11" s="10" t="s">
+      <c r="D11" s="9" t="s">
         <v>25</v>
       </c>
-      <c r="G11" s="9" t="s">
+      <c r="G11" s="8" t="s">
         <v>24</v>
       </c>
-      <c r="H11" s="10" t="s">
+      <c r="H11" s="9" t="s">
         <v>26</v>
       </c>
-      <c r="K11" s="9" t="s">
+      <c r="K11" s="8" t="s">
         <v>24</v>
       </c>
-      <c r="L11" s="10" t="s">
+      <c r="L11" s="9" t="s">
         <v>26</v>
       </c>
-      <c r="O11" s="9" t="s">
+      <c r="O11" s="8" t="s">
         <v>24</v>
       </c>
-      <c r="P11" s="10" t="s">
+      <c r="P11" s="9" t="s">
         <v>26</v>
       </c>
-      <c r="S11" s="9" t="s">
+      <c r="S11" s="8" t="s">
         <v>24</v>
       </c>
-      <c r="T11" s="10" t="s">
+      <c r="T11" s="9" t="s">
         <v>26</v>
       </c>
-      <c r="X11" s="9" t="s">
+      <c r="X11" s="8" t="s">
         <v>24</v>
       </c>
-      <c r="Y11" s="10" t="s">
+      <c r="Y11" s="9" t="s">
         <v>27</v>
       </c>
     </row>
     <row r="12" spans="1:25" x14ac:dyDescent="0.25">
-      <c r="A12" s="11" t="s">
+      <c r="A12" s="10" t="s">
         <v>28</v>
       </c>
-      <c r="B12" s="2"/>
-      <c r="C12" s="9" t="s">
+      <c r="B12" s="1"/>
+      <c r="C12" s="8" t="s">
         <v>29</v>
       </c>
-      <c r="D12" s="10" t="s">
+      <c r="D12" s="9" t="s">
         <v>25</v>
       </c>
-      <c r="G12" s="9" t="s">
+      <c r="G12" s="8" t="s">
         <v>29</v>
       </c>
-      <c r="H12" s="10" t="s">
+      <c r="H12" s="9" t="s">
         <v>30</v>
       </c>
-      <c r="K12" s="9" t="s">
+      <c r="K12" s="8" t="s">
         <v>29</v>
       </c>
-      <c r="L12" s="10" t="s">
+      <c r="L12" s="9" t="s">
         <v>26</v>
       </c>
-      <c r="O12" s="9" t="s">
+      <c r="O12" s="8" t="s">
         <v>29</v>
       </c>
-      <c r="P12" s="10" t="s">
+      <c r="P12" s="9" t="s">
         <v>26</v>
       </c>
-      <c r="S12" s="9" t="s">
+      <c r="S12" s="8" t="s">
         <v>29</v>
       </c>
-      <c r="T12" s="10" t="s">
+      <c r="T12" s="9" t="s">
         <v>26</v>
       </c>
-      <c r="X12" s="9" t="s">
+      <c r="X12" s="8" t="s">
         <v>29</v>
       </c>
-      <c r="Y12" s="10" t="s">
+      <c r="Y12" s="9" t="s">
         <v>25</v>
       </c>
     </row>
     <row r="13" spans="1:25" x14ac:dyDescent="0.25">
-      <c r="C13" s="9" t="s">
+      <c r="C13" s="8" t="s">
         <v>31</v>
       </c>
-      <c r="D13" s="10" t="s">
+      <c r="D13" s="9" t="s">
         <v>32</v>
       </c>
-      <c r="G13" s="9" t="s">
+      <c r="G13" s="8" t="s">
         <v>31</v>
       </c>
-      <c r="H13" s="10" t="s">
+      <c r="H13" s="9" t="s">
         <v>32</v>
       </c>
-      <c r="K13" s="9" t="s">
+      <c r="K13" s="8" t="s">
         <v>31</v>
       </c>
-      <c r="L13" s="10" t="s">
+      <c r="L13" s="9" t="s">
         <v>32</v>
       </c>
-      <c r="O13" s="9" t="s">
+      <c r="O13" s="8" t="s">
         <v>31</v>
       </c>
-      <c r="P13" s="10" t="s">
+      <c r="P13" s="9" t="s">
         <v>32</v>
       </c>
-      <c r="S13" s="9" t="s">
+      <c r="S13" s="8" t="s">
         <v>31</v>
       </c>
-      <c r="T13" s="10" t="s">
+      <c r="T13" s="9" t="s">
         <v>32</v>
       </c>
-      <c r="X13" s="9" t="s">
+      <c r="X13" s="8" t="s">
         <v>31</v>
       </c>
-      <c r="Y13" s="10" t="s">
+      <c r="Y13" s="9" t="s">
         <v>32</v>
       </c>
     </row>
     <row r="14" spans="1:25" ht="30" x14ac:dyDescent="0.25">
-      <c r="C14" s="12" t="s">
+      <c r="C14" s="11" t="s">
         <v>1</v>
       </c>
-      <c r="D14" s="13" t="s">
+      <c r="D14" s="12" t="s">
         <v>33</v>
       </c>
-      <c r="G14" s="12" t="s">
+      <c r="G14" s="11" t="s">
         <v>1</v>
       </c>
-      <c r="H14" s="13" t="s">
+      <c r="H14" s="12" t="s">
         <v>33</v>
       </c>
-      <c r="K14" s="12" t="s">
+      <c r="K14" s="11" t="s">
         <v>1</v>
       </c>
-      <c r="L14" s="13" t="s">
+      <c r="L14" s="12" t="s">
         <v>33</v>
       </c>
-      <c r="O14" s="12" t="s">
+      <c r="O14" s="11" t="s">
         <v>1</v>
       </c>
-      <c r="P14" s="13" t="s">
+      <c r="P14" s="12" t="s">
         <v>33</v>
       </c>
-      <c r="S14" s="12" t="s">
+      <c r="S14" s="11" t="s">
         <v>1</v>
       </c>
-      <c r="T14" s="13" t="s">
+      <c r="T14" s="12" t="s">
         <v>33</v>
       </c>
-      <c r="X14" s="12" t="s">
+      <c r="X14" s="11" t="s">
         <v>1</v>
       </c>
-      <c r="Y14" s="13" t="s">
+      <c r="Y14" s="12" t="s">
         <v>33</v>
       </c>
     </row>
     <row r="15" spans="1:25" x14ac:dyDescent="0.25">
-      <c r="C15" s="14" t="s">
+      <c r="C15" s="22" t="s">
+        <v>68</v>
+      </c>
+      <c r="D15" s="9" t="s">
+        <v>69</v>
+      </c>
+      <c r="G15" s="22" t="s">
+        <v>68</v>
+      </c>
+      <c r="H15" s="9" t="s">
+        <v>69</v>
+      </c>
+      <c r="K15" s="22" t="s">
+        <v>68</v>
+      </c>
+      <c r="L15" s="9" t="s">
+        <v>69</v>
+      </c>
+      <c r="O15" s="22" t="s">
+        <v>68</v>
+      </c>
+      <c r="P15" s="9" t="s">
+        <v>69</v>
+      </c>
+      <c r="S15" s="22" t="s">
+        <v>68</v>
+      </c>
+      <c r="T15" s="9" t="s">
+        <v>69</v>
+      </c>
+      <c r="X15" s="22" t="s">
+        <v>68</v>
+      </c>
+      <c r="Y15" s="9" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="16" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="C16" s="22" t="s">
+        <v>67</v>
+      </c>
+      <c r="D16" s="9" t="s">
+        <v>70</v>
+      </c>
+      <c r="G16" s="22" t="s">
+        <v>67</v>
+      </c>
+      <c r="H16" s="9" t="s">
+        <v>70</v>
+      </c>
+      <c r="K16" s="22" t="s">
+        <v>67</v>
+      </c>
+      <c r="L16" s="9" t="s">
+        <v>70</v>
+      </c>
+      <c r="O16" s="22" t="s">
+        <v>67</v>
+      </c>
+      <c r="P16" s="9" t="s">
+        <v>70</v>
+      </c>
+      <c r="S16" s="22" t="s">
+        <v>67</v>
+      </c>
+      <c r="T16" s="9" t="s">
+        <v>70</v>
+      </c>
+      <c r="X16" s="22" t="s">
+        <v>67</v>
+      </c>
+      <c r="Y16" s="9" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="17" spans="3:25" x14ac:dyDescent="0.25">
+      <c r="C17" s="17" t="s">
         <v>34</v>
       </c>
-      <c r="D15" s="15"/>
-      <c r="G15" s="14" t="s">
+      <c r="D17" s="18"/>
+      <c r="G17" s="17" t="s">
         <v>34</v>
       </c>
-      <c r="H15" s="15"/>
-      <c r="K15" s="14" t="s">
+      <c r="H17" s="18"/>
+      <c r="K17" s="17" t="s">
         <v>34</v>
       </c>
-      <c r="L15" s="15"/>
-      <c r="O15" s="14" t="s">
+      <c r="L17" s="18"/>
+      <c r="O17" s="17" t="s">
         <v>34</v>
       </c>
-      <c r="P15" s="15"/>
-      <c r="S15" s="14" t="s">
+      <c r="P17" s="18"/>
+      <c r="S17" s="17" t="s">
         <v>34</v>
       </c>
-      <c r="T15" s="15"/>
-      <c r="X15" s="14" t="s">
+      <c r="T17" s="18"/>
+      <c r="X17" s="17" t="s">
         <v>34</v>
       </c>
-      <c r="Y15" s="15"/>
-    </row>
-    <row r="16" spans="1:25" ht="90" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C16" s="16" t="s">
+      <c r="Y17" s="18"/>
+    </row>
+    <row r="18" spans="3:25" ht="90" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C18" s="13" t="s">
         <v>35</v>
       </c>
-      <c r="D16" s="17"/>
-      <c r="G16" s="16" t="s">
+      <c r="D18" s="14"/>
+      <c r="G18" s="13" t="s">
         <v>36</v>
       </c>
-      <c r="H16" s="17"/>
-      <c r="K16" s="16" t="s">
+      <c r="H18" s="14"/>
+      <c r="K18" s="13" t="s">
         <v>37</v>
       </c>
-      <c r="L16" s="17"/>
-      <c r="O16" s="16" t="s">
+      <c r="L18" s="14"/>
+      <c r="O18" s="13" t="s">
         <v>38</v>
       </c>
-      <c r="P16" s="17"/>
-      <c r="S16" s="16" t="s">
+      <c r="P18" s="14"/>
+      <c r="S18" s="13" t="s">
         <v>39</v>
       </c>
-      <c r="T16" s="17"/>
-      <c r="X16" s="16" t="s">
+      <c r="T18" s="14"/>
+      <c r="X18" s="13" t="s">
         <v>40</v>
       </c>
-      <c r="Y16" s="17"/>
-    </row>
-    <row r="17" spans="3:25" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C17" s="14" t="s">
+      <c r="Y18" s="14"/>
+    </row>
+    <row r="19" spans="3:25" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C19" s="17" t="s">
         <v>41</v>
       </c>
-      <c r="D17" s="15"/>
-      <c r="G17" s="14" t="s">
+      <c r="D19" s="18"/>
+      <c r="G19" s="17" t="s">
         <v>41</v>
       </c>
-      <c r="H17" s="15"/>
-      <c r="K17" s="14" t="s">
+      <c r="H19" s="18"/>
+      <c r="K19" s="17" t="s">
         <v>41</v>
       </c>
-      <c r="L17" s="15"/>
-      <c r="O17" s="14" t="s">
+      <c r="L19" s="18"/>
+      <c r="O19" s="17" t="s">
         <v>41</v>
       </c>
-      <c r="P17" s="15"/>
-      <c r="S17" s="14" t="s">
+      <c r="P19" s="18"/>
+      <c r="S19" s="17" t="s">
         <v>41</v>
       </c>
-      <c r="T17" s="15"/>
-      <c r="X17" s="14" t="s">
+      <c r="T19" s="18"/>
+      <c r="X19" s="17" t="s">
         <v>41</v>
       </c>
-      <c r="Y17" s="15"/>
-    </row>
-    <row r="18" spans="3:25" ht="123" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C18" s="18" t="s">
+      <c r="Y19" s="18"/>
+    </row>
+    <row r="20" spans="3:25" ht="123" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C20" s="19" t="s">
         <v>42</v>
       </c>
-      <c r="D18" s="19"/>
-      <c r="G18" s="18" t="s">
+      <c r="D20" s="20"/>
+      <c r="G20" s="19" t="s">
         <v>43</v>
       </c>
-      <c r="H18" s="19"/>
-      <c r="K18" s="18" t="s">
+      <c r="H20" s="20"/>
+      <c r="K20" s="19" t="s">
         <v>44</v>
       </c>
-      <c r="L18" s="19"/>
-      <c r="O18" s="18" t="s">
+      <c r="L20" s="20"/>
+      <c r="O20" s="19" t="s">
         <v>45</v>
       </c>
-      <c r="P18" s="19"/>
-      <c r="S18" s="18" t="s">
+      <c r="P20" s="20"/>
+      <c r="S20" s="19" t="s">
         <v>46</v>
       </c>
-      <c r="T18" s="19"/>
-      <c r="X18" s="18" t="s">
+      <c r="T20" s="20"/>
+      <c r="X20" s="19" t="s">
         <v>47</v>
       </c>
-      <c r="Y18" s="19"/>
-    </row>
-    <row r="19" spans="3:25" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C19" s="14" t="s">
+      <c r="Y20" s="20"/>
+    </row>
+    <row r="21" spans="3:25" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C21" s="17" t="s">
         <v>48</v>
       </c>
-      <c r="D19" s="15"/>
-      <c r="G19" s="14" t="s">
+      <c r="D21" s="18"/>
+      <c r="G21" s="17" t="s">
         <v>48</v>
       </c>
-      <c r="H19" s="15"/>
-      <c r="K19" s="14" t="s">
+      <c r="H21" s="18"/>
+      <c r="K21" s="17" t="s">
         <v>48</v>
       </c>
-      <c r="L19" s="15"/>
-      <c r="O19" s="14" t="s">
+      <c r="L21" s="18"/>
+      <c r="O21" s="17" t="s">
         <v>48</v>
       </c>
-      <c r="P19" s="15"/>
-      <c r="S19" s="14" t="s">
+      <c r="P21" s="18"/>
+      <c r="S21" s="17" t="s">
         <v>48</v>
       </c>
-      <c r="T19" s="15"/>
-      <c r="X19" s="14" t="s">
+      <c r="T21" s="18"/>
+      <c r="X21" s="17" t="s">
         <v>48</v>
       </c>
-      <c r="Y19" s="15"/>
-    </row>
-    <row r="20" spans="3:25" ht="126.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C20" s="16" t="s">
+      <c r="Y21" s="18"/>
+    </row>
+    <row r="22" spans="3:25" ht="126.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C22" s="13" t="s">
         <v>49</v>
       </c>
-      <c r="D20" s="17"/>
-      <c r="G20" s="16" t="s">
+      <c r="D22" s="14"/>
+      <c r="G22" s="13" t="s">
         <v>50</v>
       </c>
-      <c r="H20" s="17"/>
-      <c r="K20" s="16" t="s">
+      <c r="H22" s="14"/>
+      <c r="K22" s="13" t="s">
         <v>51</v>
       </c>
-      <c r="L20" s="17"/>
-      <c r="O20" s="16" t="s">
+      <c r="L22" s="14"/>
+      <c r="O22" s="13" t="s">
         <v>52</v>
       </c>
-      <c r="P20" s="17"/>
-      <c r="S20" s="16" t="s">
+      <c r="P22" s="14"/>
+      <c r="S22" s="13" t="s">
         <v>53</v>
       </c>
-      <c r="T20" s="17"/>
-      <c r="X20" s="16" t="s">
+      <c r="T22" s="14"/>
+      <c r="X22" s="13" t="s">
         <v>54</v>
       </c>
-      <c r="Y20" s="17"/>
-    </row>
-    <row r="21" spans="3:25" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C21" s="14" t="s">
+      <c r="Y22" s="14"/>
+    </row>
+    <row r="23" spans="3:25" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C23" s="17" t="s">
         <v>55</v>
       </c>
-      <c r="D21" s="15"/>
-      <c r="G21" s="14" t="s">
+      <c r="D23" s="18"/>
+      <c r="G23" s="17" t="s">
         <v>55</v>
       </c>
-      <c r="H21" s="15"/>
-      <c r="K21" s="14" t="s">
+      <c r="H23" s="18"/>
+      <c r="K23" s="17" t="s">
         <v>55</v>
       </c>
-      <c r="L21" s="15"/>
-      <c r="O21" s="14" t="s">
+      <c r="L23" s="18"/>
+      <c r="O23" s="17" t="s">
         <v>55</v>
       </c>
-      <c r="P21" s="15"/>
-      <c r="S21" s="14" t="s">
+      <c r="P23" s="18"/>
+      <c r="S23" s="17" t="s">
         <v>55</v>
       </c>
-      <c r="T21" s="15"/>
-      <c r="X21" s="14" t="s">
+      <c r="T23" s="18"/>
+      <c r="X23" s="17" t="s">
         <v>55</v>
       </c>
-      <c r="Y21" s="15"/>
-    </row>
-    <row r="22" spans="3:25" ht="113.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C22" s="16" t="s">
+      <c r="Y23" s="18"/>
+    </row>
+    <row r="24" spans="3:25" ht="113.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C24" s="13" t="s">
         <v>56</v>
       </c>
-      <c r="D22" s="17"/>
-      <c r="G22" s="16" t="s">
+      <c r="D24" s="14"/>
+      <c r="G24" s="13" t="s">
         <v>57</v>
       </c>
-      <c r="H22" s="17"/>
-      <c r="K22" s="16" t="s">
+      <c r="H24" s="14"/>
+      <c r="K24" s="13" t="s">
         <v>58</v>
       </c>
-      <c r="L22" s="17"/>
-      <c r="O22" s="16" t="s">
+      <c r="L24" s="14"/>
+      <c r="O24" s="13" t="s">
         <v>59</v>
       </c>
-      <c r="P22" s="17"/>
-      <c r="S22" s="16" t="s">
+      <c r="P24" s="14"/>
+      <c r="S24" s="13" t="s">
         <v>60</v>
       </c>
-      <c r="T22" s="17"/>
-      <c r="X22" s="16" t="s">
+      <c r="T24" s="14"/>
+      <c r="X24" s="13" t="s">
         <v>61</v>
       </c>
-      <c r="Y22" s="17"/>
-    </row>
-    <row r="23" spans="3:25" x14ac:dyDescent="0.25">
-      <c r="C23" s="14" t="s">
+      <c r="Y24" s="14"/>
+    </row>
+    <row r="25" spans="3:25" x14ac:dyDescent="0.25">
+      <c r="C25" s="17" t="s">
         <v>62</v>
       </c>
-      <c r="D23" s="15"/>
-      <c r="G23" s="14" t="s">
+      <c r="D25" s="18"/>
+      <c r="G25" s="17" t="s">
         <v>62</v>
       </c>
-      <c r="H23" s="15"/>
-      <c r="K23" s="14" t="s">
+      <c r="H25" s="18"/>
+      <c r="K25" s="17" t="s">
         <v>62</v>
       </c>
-      <c r="L23" s="15"/>
-      <c r="O23" s="14" t="s">
+      <c r="L25" s="18"/>
+      <c r="O25" s="17" t="s">
         <v>62</v>
       </c>
-      <c r="P23" s="15"/>
-      <c r="S23" s="14" t="s">
+      <c r="P25" s="18"/>
+      <c r="S25" s="17" t="s">
         <v>62</v>
       </c>
-      <c r="T23" s="15"/>
-      <c r="X23" s="14" t="s">
+      <c r="T25" s="18"/>
+      <c r="X25" s="17" t="s">
         <v>62</v>
       </c>
-      <c r="Y23" s="15"/>
-    </row>
-    <row r="24" spans="3:25" ht="247.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C24" s="16"/>
-      <c r="D24" s="17"/>
-      <c r="G24" s="20" t="s">
+      <c r="Y25" s="18"/>
+    </row>
+    <row r="26" spans="3:25" ht="247.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C26" s="13"/>
+      <c r="D26" s="14"/>
+      <c r="G26" s="15" t="s">
         <v>63</v>
       </c>
-      <c r="H24" s="21"/>
-      <c r="K24" s="20" t="s">
+      <c r="H26" s="16"/>
+      <c r="K26" s="15" t="s">
         <v>64</v>
       </c>
-      <c r="L24" s="21"/>
-      <c r="O24" s="20" t="s">
+      <c r="L26" s="16"/>
+      <c r="O26" s="15" t="s">
         <v>65</v>
       </c>
-      <c r="P24" s="21"/>
-      <c r="S24" s="16" t="s">
+      <c r="P26" s="16"/>
+      <c r="S26" s="13" t="s">
         <v>66</v>
       </c>
-      <c r="T24" s="17"/>
-      <c r="X24" s="16"/>
-      <c r="Y24" s="17"/>
+      <c r="T26" s="14"/>
+      <c r="X26" s="13"/>
+      <c r="Y26" s="14"/>
     </row>
   </sheetData>
   <mergeCells count="61">
-    <mergeCell ref="C24:D24"/>
-    <mergeCell ref="G24:H24"/>
-    <mergeCell ref="K24:L24"/>
-    <mergeCell ref="O24:P24"/>
-    <mergeCell ref="S24:T24"/>
+    <mergeCell ref="A2:C2"/>
+    <mergeCell ref="C17:D17"/>
+    <mergeCell ref="G17:H17"/>
+    <mergeCell ref="K17:L17"/>
+    <mergeCell ref="O17:P17"/>
+    <mergeCell ref="X17:Y17"/>
+    <mergeCell ref="C18:D18"/>
+    <mergeCell ref="G18:H18"/>
+    <mergeCell ref="K18:L18"/>
+    <mergeCell ref="O18:P18"/>
+    <mergeCell ref="S18:T18"/>
+    <mergeCell ref="X18:Y18"/>
+    <mergeCell ref="S17:T17"/>
+    <mergeCell ref="X20:Y20"/>
+    <mergeCell ref="C19:D19"/>
+    <mergeCell ref="G19:H19"/>
+    <mergeCell ref="K19:L19"/>
+    <mergeCell ref="O19:P19"/>
+    <mergeCell ref="S19:T19"/>
+    <mergeCell ref="X19:Y19"/>
+    <mergeCell ref="C20:D20"/>
+    <mergeCell ref="G20:H20"/>
+    <mergeCell ref="K20:L20"/>
+    <mergeCell ref="O20:P20"/>
+    <mergeCell ref="S20:T20"/>
+    <mergeCell ref="X22:Y22"/>
+    <mergeCell ref="C21:D21"/>
+    <mergeCell ref="G21:H21"/>
+    <mergeCell ref="K21:L21"/>
+    <mergeCell ref="O21:P21"/>
+    <mergeCell ref="S21:T21"/>
+    <mergeCell ref="X21:Y21"/>
+    <mergeCell ref="C22:D22"/>
+    <mergeCell ref="G22:H22"/>
+    <mergeCell ref="K22:L22"/>
+    <mergeCell ref="O22:P22"/>
+    <mergeCell ref="S22:T22"/>
     <mergeCell ref="X24:Y24"/>
     <mergeCell ref="C23:D23"/>
     <mergeCell ref="G23:H23"/>
@@ -1711,55 +1845,23 @@
     <mergeCell ref="O23:P23"/>
     <mergeCell ref="S23:T23"/>
     <mergeCell ref="X23:Y23"/>
-    <mergeCell ref="C22:D22"/>
-    <mergeCell ref="G22:H22"/>
-    <mergeCell ref="K22:L22"/>
-    <mergeCell ref="O22:P22"/>
-    <mergeCell ref="S22:T22"/>
-    <mergeCell ref="X22:Y22"/>
-    <mergeCell ref="C21:D21"/>
-    <mergeCell ref="G21:H21"/>
-    <mergeCell ref="K21:L21"/>
-    <mergeCell ref="O21:P21"/>
-    <mergeCell ref="S21:T21"/>
-    <mergeCell ref="X21:Y21"/>
-    <mergeCell ref="C20:D20"/>
-    <mergeCell ref="G20:H20"/>
-    <mergeCell ref="K20:L20"/>
-    <mergeCell ref="O20:P20"/>
-    <mergeCell ref="S20:T20"/>
-    <mergeCell ref="X20:Y20"/>
-    <mergeCell ref="C19:D19"/>
-    <mergeCell ref="G19:H19"/>
-    <mergeCell ref="K19:L19"/>
-    <mergeCell ref="O19:P19"/>
-    <mergeCell ref="S19:T19"/>
-    <mergeCell ref="X19:Y19"/>
-    <mergeCell ref="C18:D18"/>
-    <mergeCell ref="G18:H18"/>
-    <mergeCell ref="K18:L18"/>
-    <mergeCell ref="O18:P18"/>
-    <mergeCell ref="S18:T18"/>
-    <mergeCell ref="X18:Y18"/>
-    <mergeCell ref="C17:D17"/>
-    <mergeCell ref="G17:H17"/>
-    <mergeCell ref="K17:L17"/>
-    <mergeCell ref="O17:P17"/>
-    <mergeCell ref="S17:T17"/>
-    <mergeCell ref="X17:Y17"/>
-    <mergeCell ref="X15:Y15"/>
-    <mergeCell ref="C16:D16"/>
-    <mergeCell ref="G16:H16"/>
-    <mergeCell ref="K16:L16"/>
-    <mergeCell ref="O16:P16"/>
-    <mergeCell ref="S16:T16"/>
-    <mergeCell ref="X16:Y16"/>
-    <mergeCell ref="A2:C2"/>
-    <mergeCell ref="C15:D15"/>
-    <mergeCell ref="G15:H15"/>
-    <mergeCell ref="K15:L15"/>
-    <mergeCell ref="O15:P15"/>
-    <mergeCell ref="S15:T15"/>
+    <mergeCell ref="C24:D24"/>
+    <mergeCell ref="G24:H24"/>
+    <mergeCell ref="K24:L24"/>
+    <mergeCell ref="O24:P24"/>
+    <mergeCell ref="S24:T24"/>
+    <mergeCell ref="X26:Y26"/>
+    <mergeCell ref="C25:D25"/>
+    <mergeCell ref="G25:H25"/>
+    <mergeCell ref="K25:L25"/>
+    <mergeCell ref="O25:P25"/>
+    <mergeCell ref="S25:T25"/>
+    <mergeCell ref="X25:Y25"/>
+    <mergeCell ref="C26:D26"/>
+    <mergeCell ref="G26:H26"/>
+    <mergeCell ref="K26:L26"/>
+    <mergeCell ref="O26:P26"/>
+    <mergeCell ref="S26:T26"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>

</xml_diff>